<commit_message>
run for 2025 update
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="270">
   <si>
     <t>TileID</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Community</t>
   </si>
   <si>
-    <t>Region</t>
-  </si>
-  <si>
     <t>Delaware County</t>
   </si>
   <si>
@@ -112,6 +109,12 @@
     <t>Union County</t>
   </si>
   <si>
+    <t>Ashville</t>
+  </si>
+  <si>
+    <t>Baltimore</t>
+  </si>
+  <si>
     <t>Bloom Township (Fairfield)</t>
   </si>
   <si>
@@ -157,36 +160,33 @@
     <t>Washington Township (Franklin)</t>
   </si>
   <si>
+    <t>Bellefontaine</t>
+  </si>
+  <si>
+    <t>Bexley</t>
+  </si>
+  <si>
     <t>Etna Township (Licking)</t>
   </si>
   <si>
     <t>Granville Township (Licking)</t>
   </si>
   <si>
+    <t>Buckeye Lake</t>
+  </si>
+  <si>
+    <t>Canal Winchester</t>
+  </si>
+  <si>
+    <t>Chillicothe</t>
+  </si>
+  <si>
+    <t>Circleville</t>
+  </si>
+  <si>
     <t>Jerome Township (Union)</t>
   </si>
   <si>
-    <t>Ashville</t>
-  </si>
-  <si>
-    <t>Bellefontaine</t>
-  </si>
-  <si>
-    <t>Bexley</t>
-  </si>
-  <si>
-    <t>Buckeye Lake</t>
-  </si>
-  <si>
-    <t>Canal Winchester</t>
-  </si>
-  <si>
-    <t>Chillicothe</t>
-  </si>
-  <si>
-    <t>Circleville</t>
-  </si>
-  <si>
     <t>Columbus</t>
   </si>
   <si>
@@ -313,9 +313,6 @@
     <t>Worthington</t>
   </si>
   <si>
-    <t>15-County Region</t>
-  </si>
-  <si>
     <t>TBD</t>
   </si>
   <si>
@@ -364,208 +361,208 @@
     <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0500000US39159.svg</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390450695099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390458020699999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390490692299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390490944299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390491611299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390492828099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390493777299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390493861299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390494641099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390495006499999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390496184099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390496297499999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390496457099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390497771499999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390498124299999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390892569099999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US390893141699999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/0700000US391593904699999.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3902680.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3905130.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3906278.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3909890.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3911332.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3914184.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3915070.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3918000.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3921434.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3922694.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3929106.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3929148.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3931304.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3931402.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3932592.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3932606.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3934748.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3934790.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3935476.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3939340.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3941720.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3944086.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3944674.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3947474.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3947754.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3948160.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3950862.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3953046.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3953102.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3953970.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3954040.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3954866.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3957862.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3961112.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3962498.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3963030.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3964486.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3966390.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3967440.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3971976.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3972977.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3973068.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3975602.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3979002.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3979100.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3983342.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3983580.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3984742.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/1600000US3986604.svg</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M010000US001.svg</t>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3902680.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3903758.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390450695099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390458020699999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390490692299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390490944299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390491611299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390492828099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390493777299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390493861299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390494641099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390495006499999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390496184099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390496297499999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390496457099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390497771499999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390498124299999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3905130.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3906278.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390892569099999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US390893141699999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3909890.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3911332.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3914184.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3915070.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US391593904699999.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3918000.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3921434.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3922694.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3929106.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3929148.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3931304.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3931402.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3932592.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3932606.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3934748.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3934790.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3935476.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3939340.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3941720.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3944086.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3944674.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3947474.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3947754.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3948160.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3950862.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3953046.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3953102.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3953970.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3954040.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3954866.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3957862.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3961112.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3962498.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3963030.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3964486.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3966390.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3967440.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3971976.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3972977.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3973068.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3975602.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3979002.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3979100.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3983342.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3983580.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3984742.svg</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/morpc-insights/insights-housingprice/refs/heads/main/output_data/charts/M100000US3986604.svg</t>
   </si>
   <si>
     <t>Mid-Ohio Regional Planning Commission</t>
@@ -622,208 +619,208 @@
     <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0500000US39159</t>
   </si>
   <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390450695099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390458020699999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390490692299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390490944299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390491611299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390492828099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390493777299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390493861299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390494641099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390495006499999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390496184099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390496297499999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390496457099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390497771499999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390498124299999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390892569099999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US390893141699999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=0700000US391593904699999</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3902680</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3905130</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3906278</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3909890</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3911332</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3914184</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3915070</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3918000</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3921434</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3922694</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3929106</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3929148</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3931304</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3931402</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3932592</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3932606</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3934748</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3934790</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3935476</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3939340</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3941720</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3944086</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3944674</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3947474</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3947754</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3948160</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3950862</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3953046</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3953102</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3953970</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3954040</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3954866</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3957862</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3961112</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3962498</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3963030</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3964486</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3966390</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3967440</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3971976</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3972977</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3973068</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3975602</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3979002</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3979100</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3983342</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3983580</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3984742</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=1600000US3986604</t>
-  </si>
-  <si>
-    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M010000US001</t>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3902680</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3903758</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390450695099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390458020699999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390490692299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390490944299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390491611299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390492828099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390493777299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390493861299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390494641099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390495006499999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390496184099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390496297499999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390496457099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390497771499999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390498124299999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3905130</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3906278</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390892569099999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US390893141699999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3909890</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3911332</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3914184</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3915070</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US391593904699999</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3918000</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3921434</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3922694</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3929106</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3929148</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3931304</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3931402</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3932592</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3932606</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3934748</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3934790</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3935476</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3939340</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3941720</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3944086</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3944674</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3947474</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3947754</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3948160</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3950862</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3953046</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3953102</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3953970</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3954040</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3954866</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3957862</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3961112</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3962498</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3963030</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3964486</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3966390</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3967440</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3971976</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3972977</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3973068</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3975602</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3979002</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3979100</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3983342</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3983580</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3984742</t>
+  </si>
+  <si>
+    <t>https://www.arcgis.com/apps/dashboards/237dd7c3dc694feebe0b3e6381f45f93#geoid=M100000US3986604</t>
   </si>
   <si>
     <t>https://morpc1-my.sharepoint.com/:w:/g/personal/aporr_morpc_org/EeowBvR-mvJEsEDFbiSWb1kBE5DcjowKjyYzzKE35vwfwg?e=KCvIsQ</t>
@@ -1249,31 +1246,31 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G2" t="s">
-        <v>100</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="I2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>187</v>
-      </c>
       <c r="N2" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:14">
@@ -1281,31 +1278,31 @@
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1313,31 +1310,31 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -1345,31 +1342,31 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -1377,31 +1374,31 @@
         <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -1409,31 +1406,31 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -1441,31 +1438,31 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -1473,31 +1470,31 @@
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -1505,31 +1502,31 @@
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -1537,31 +1534,31 @@
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1569,31 +1566,31 @@
         <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -1601,31 +1598,31 @@
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -1633,31 +1630,31 @@
         <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -1665,31 +1662,31 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="I15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -1697,31 +1694,31 @@
         <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" spans="3:14">
@@ -1729,31 +1726,31 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="3:14">
@@ -1761,511 +1758,466 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I18" t="s">
+        <v>183</v>
+      </c>
+      <c r="J18" t="s">
+        <v>184</v>
+      </c>
+      <c r="K18" t="s">
+        <v>185</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="3:14">
+      <c r="D19" t="s">
         <v>33</v>
       </c>
-      <c r="F18" t="s">
-        <v>100</v>
-      </c>
-      <c r="G18" t="s">
-        <v>100</v>
-      </c>
-      <c r="H18" s="2" t="s">
+      <c r="F19" t="s">
+        <v>99</v>
+      </c>
+      <c r="G19" t="s">
+        <v>99</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I18" t="s">
-        <v>184</v>
-      </c>
-      <c r="J18" t="s">
-        <v>185</v>
-      </c>
-      <c r="K18" t="s">
-        <v>186</v>
-      </c>
-      <c r="M18" s="2" t="s">
+      <c r="I19" t="s">
+        <v>183</v>
+      </c>
+      <c r="J19" t="s">
+        <v>184</v>
+      </c>
+      <c r="K19" t="s">
+        <v>185</v>
+      </c>
+      <c r="M19" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="N18" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19" spans="3:14">
-      <c r="C19" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="N19" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="20" spans="3:14">
+      <c r="D20" t="s">
         <v>34</v>
       </c>
-      <c r="F19" t="s">
-        <v>100</v>
-      </c>
-      <c r="G19" t="s">
-        <v>100</v>
-      </c>
-      <c r="H19" s="2" t="s">
+      <c r="F20" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="I19" t="s">
-        <v>184</v>
-      </c>
-      <c r="J19" t="s">
-        <v>185</v>
-      </c>
-      <c r="K19" t="s">
-        <v>186</v>
-      </c>
-      <c r="M19" s="2" t="s">
+      <c r="I20" t="s">
+        <v>183</v>
+      </c>
+      <c r="J20" t="s">
+        <v>184</v>
+      </c>
+      <c r="K20" t="s">
+        <v>185</v>
+      </c>
+      <c r="M20" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="N19" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="20" spans="3:14">
-      <c r="C20" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="N20" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="21" spans="3:14">
+      <c r="D21" t="s">
         <v>35</v>
       </c>
-      <c r="F20" t="s">
-        <v>100</v>
-      </c>
-      <c r="G20" t="s">
-        <v>100</v>
-      </c>
-      <c r="H20" s="2" t="s">
+      <c r="F21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G21" t="s">
+        <v>99</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I20" t="s">
-        <v>184</v>
-      </c>
-      <c r="J20" t="s">
-        <v>185</v>
-      </c>
-      <c r="K20" t="s">
-        <v>186</v>
-      </c>
-      <c r="M20" s="2" t="s">
+      <c r="I21" t="s">
+        <v>183</v>
+      </c>
+      <c r="J21" t="s">
+        <v>184</v>
+      </c>
+      <c r="K21" t="s">
+        <v>185</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="N20" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="21" spans="3:14">
-      <c r="C21" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="N21" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="22" spans="3:14">
+      <c r="D22" t="s">
         <v>36</v>
       </c>
-      <c r="F21" t="s">
-        <v>100</v>
-      </c>
-      <c r="G21" t="s">
-        <v>100</v>
-      </c>
-      <c r="H21" s="2" t="s">
+      <c r="F22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22" t="s">
+        <v>99</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="I21" t="s">
-        <v>184</v>
-      </c>
-      <c r="J21" t="s">
-        <v>185</v>
-      </c>
-      <c r="K21" t="s">
-        <v>186</v>
-      </c>
-      <c r="M21" s="2" t="s">
+      <c r="I22" t="s">
+        <v>183</v>
+      </c>
+      <c r="J22" t="s">
+        <v>184</v>
+      </c>
+      <c r="K22" t="s">
+        <v>185</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="N21" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="22" spans="3:14">
-      <c r="C22" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="N22" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="23" spans="3:14">
+      <c r="D23" t="s">
         <v>37</v>
       </c>
-      <c r="F22" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22" t="s">
-        <v>100</v>
-      </c>
-      <c r="H22" s="2" t="s">
+      <c r="F23" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="I22" t="s">
-        <v>184</v>
-      </c>
-      <c r="J22" t="s">
-        <v>185</v>
-      </c>
-      <c r="K22" t="s">
-        <v>186</v>
-      </c>
-      <c r="M22" s="2" t="s">
+      <c r="I23" t="s">
+        <v>183</v>
+      </c>
+      <c r="J23" t="s">
+        <v>184</v>
+      </c>
+      <c r="K23" t="s">
+        <v>185</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="N22" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="23" spans="3:14">
-      <c r="C23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="N23" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="24" spans="3:14">
+      <c r="D24" t="s">
         <v>38</v>
       </c>
-      <c r="F23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G23" t="s">
-        <v>100</v>
-      </c>
-      <c r="H23" s="2" t="s">
+      <c r="F24" t="s">
+        <v>99</v>
+      </c>
+      <c r="G24" t="s">
+        <v>99</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I23" t="s">
-        <v>184</v>
-      </c>
-      <c r="J23" t="s">
-        <v>185</v>
-      </c>
-      <c r="K23" t="s">
-        <v>186</v>
-      </c>
-      <c r="M23" s="2" t="s">
+      <c r="I24" t="s">
+        <v>183</v>
+      </c>
+      <c r="J24" t="s">
+        <v>184</v>
+      </c>
+      <c r="K24" t="s">
+        <v>185</v>
+      </c>
+      <c r="M24" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="N23" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="24" spans="3:14">
-      <c r="C24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="N24" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="25" spans="3:14">
+      <c r="D25" t="s">
         <v>39</v>
       </c>
-      <c r="F24" t="s">
-        <v>100</v>
-      </c>
-      <c r="G24" t="s">
-        <v>100</v>
-      </c>
-      <c r="H24" s="2" t="s">
+      <c r="F25" t="s">
+        <v>99</v>
+      </c>
+      <c r="G25" t="s">
+        <v>99</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I24" t="s">
-        <v>184</v>
-      </c>
-      <c r="J24" t="s">
-        <v>185</v>
-      </c>
-      <c r="K24" t="s">
-        <v>186</v>
-      </c>
-      <c r="M24" s="2" t="s">
+      <c r="I25" t="s">
+        <v>183</v>
+      </c>
+      <c r="J25" t="s">
+        <v>184</v>
+      </c>
+      <c r="K25" t="s">
+        <v>185</v>
+      </c>
+      <c r="M25" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="N24" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="25" spans="3:14">
-      <c r="C25" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="N25" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="26" spans="3:14">
+      <c r="D26" t="s">
         <v>40</v>
       </c>
-      <c r="F25" t="s">
-        <v>100</v>
-      </c>
-      <c r="G25" t="s">
-        <v>100</v>
-      </c>
-      <c r="H25" s="2" t="s">
+      <c r="F26" t="s">
+        <v>99</v>
+      </c>
+      <c r="G26" t="s">
+        <v>99</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="I25" t="s">
-        <v>184</v>
-      </c>
-      <c r="J25" t="s">
-        <v>185</v>
-      </c>
-      <c r="K25" t="s">
-        <v>186</v>
-      </c>
-      <c r="M25" s="2" t="s">
+      <c r="I26" t="s">
+        <v>183</v>
+      </c>
+      <c r="J26" t="s">
+        <v>184</v>
+      </c>
+      <c r="K26" t="s">
+        <v>185</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="N25" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="26" spans="3:14">
-      <c r="C26" t="s">
-        <v>15</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="N26" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="27" spans="3:14">
+      <c r="D27" t="s">
         <v>41</v>
       </c>
-      <c r="F26" t="s">
-        <v>100</v>
-      </c>
-      <c r="G26" t="s">
-        <v>100</v>
-      </c>
-      <c r="H26" s="2" t="s">
+      <c r="F27" t="s">
+        <v>99</v>
+      </c>
+      <c r="G27" t="s">
+        <v>99</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="I26" t="s">
-        <v>184</v>
-      </c>
-      <c r="J26" t="s">
-        <v>185</v>
-      </c>
-      <c r="K26" t="s">
-        <v>186</v>
-      </c>
-      <c r="M26" s="2" t="s">
+      <c r="I27" t="s">
+        <v>183</v>
+      </c>
+      <c r="J27" t="s">
+        <v>184</v>
+      </c>
+      <c r="K27" t="s">
+        <v>185</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="N26" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="27" spans="3:14">
-      <c r="C27" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="N27" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="28" spans="3:14">
+      <c r="D28" t="s">
         <v>42</v>
       </c>
-      <c r="F27" t="s">
-        <v>100</v>
-      </c>
-      <c r="G27" t="s">
-        <v>100</v>
-      </c>
-      <c r="H27" s="2" t="s">
+      <c r="F28" t="s">
+        <v>99</v>
+      </c>
+      <c r="G28" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="I27" t="s">
-        <v>184</v>
-      </c>
-      <c r="J27" t="s">
-        <v>185</v>
-      </c>
-      <c r="K27" t="s">
-        <v>186</v>
-      </c>
-      <c r="M27" s="2" t="s">
+      <c r="I28" t="s">
+        <v>183</v>
+      </c>
+      <c r="J28" t="s">
+        <v>184</v>
+      </c>
+      <c r="K28" t="s">
+        <v>185</v>
+      </c>
+      <c r="M28" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="N27" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="28" spans="3:14">
-      <c r="C28" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="N28" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="29" spans="3:14">
+      <c r="D29" t="s">
         <v>43</v>
       </c>
-      <c r="F28" t="s">
-        <v>100</v>
-      </c>
-      <c r="G28" t="s">
-        <v>100</v>
-      </c>
-      <c r="H28" s="2" t="s">
+      <c r="F29" t="s">
+        <v>99</v>
+      </c>
+      <c r="G29" t="s">
+        <v>99</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="I28" t="s">
-        <v>184</v>
-      </c>
-      <c r="J28" t="s">
-        <v>185</v>
-      </c>
-      <c r="K28" t="s">
-        <v>186</v>
-      </c>
-      <c r="M28" s="2" t="s">
+      <c r="I29" t="s">
+        <v>183</v>
+      </c>
+      <c r="J29" t="s">
+        <v>184</v>
+      </c>
+      <c r="K29" t="s">
+        <v>185</v>
+      </c>
+      <c r="M29" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="N28" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="29" spans="3:14">
-      <c r="C29" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="N29" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="30" spans="3:14">
+      <c r="D30" t="s">
         <v>44</v>
       </c>
-      <c r="F29" t="s">
-        <v>100</v>
-      </c>
-      <c r="G29" t="s">
-        <v>100</v>
-      </c>
-      <c r="H29" s="2" t="s">
+      <c r="F30" t="s">
+        <v>99</v>
+      </c>
+      <c r="G30" t="s">
+        <v>99</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I29" t="s">
-        <v>184</v>
-      </c>
-      <c r="J29" t="s">
-        <v>185</v>
-      </c>
-      <c r="K29" t="s">
-        <v>186</v>
-      </c>
-      <c r="M29" s="2" t="s">
+      <c r="I30" t="s">
+        <v>183</v>
+      </c>
+      <c r="J30" t="s">
+        <v>184</v>
+      </c>
+      <c r="K30" t="s">
+        <v>185</v>
+      </c>
+      <c r="M30" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="N29" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="30" spans="3:14">
-      <c r="C30" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="N30" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="31" spans="3:14">
+      <c r="D31" t="s">
         <v>45</v>
       </c>
-      <c r="F30" t="s">
-        <v>100</v>
-      </c>
-      <c r="G30" t="s">
-        <v>100</v>
-      </c>
-      <c r="H30" s="2" t="s">
+      <c r="F31" t="s">
+        <v>99</v>
+      </c>
+      <c r="G31" t="s">
+        <v>99</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="I30" t="s">
-        <v>184</v>
-      </c>
-      <c r="J30" t="s">
-        <v>185</v>
-      </c>
-      <c r="K30" t="s">
-        <v>186</v>
-      </c>
-      <c r="M30" s="2" t="s">
+      <c r="I31" t="s">
+        <v>183</v>
+      </c>
+      <c r="J31" t="s">
+        <v>184</v>
+      </c>
+      <c r="K31" t="s">
+        <v>185</v>
+      </c>
+      <c r="M31" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="N30" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="31" spans="3:14">
-      <c r="C31" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="N31" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="32" spans="3:14">
+      <c r="D32" t="s">
         <v>46</v>
       </c>
-      <c r="F31" t="s">
-        <v>100</v>
-      </c>
-      <c r="G31" t="s">
-        <v>100</v>
-      </c>
-      <c r="H31" s="2" t="s">
+      <c r="F32" t="s">
+        <v>99</v>
+      </c>
+      <c r="G32" t="s">
+        <v>99</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="I31" t="s">
-        <v>184</v>
-      </c>
-      <c r="J31" t="s">
-        <v>185</v>
-      </c>
-      <c r="K31" t="s">
-        <v>186</v>
-      </c>
-      <c r="M31" s="2" t="s">
+      <c r="I32" t="s">
+        <v>183</v>
+      </c>
+      <c r="J32" t="s">
+        <v>184</v>
+      </c>
+      <c r="K32" t="s">
+        <v>185</v>
+      </c>
+      <c r="M32" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="N31" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="32" spans="3:14">
-      <c r="C32" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="N32" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="33" spans="3:14">
+      <c r="D33" t="s">
         <v>47</v>
       </c>
-      <c r="F32" t="s">
-        <v>100</v>
-      </c>
-      <c r="G32" t="s">
-        <v>100</v>
-      </c>
-      <c r="H32" s="2" t="s">
+      <c r="F33" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" t="s">
+        <v>99</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I32" t="s">
-        <v>184</v>
-      </c>
-      <c r="J32" t="s">
-        <v>185</v>
-      </c>
-      <c r="K32" t="s">
-        <v>186</v>
-      </c>
-      <c r="M32" s="2" t="s">
+      <c r="I33" t="s">
+        <v>183</v>
+      </c>
+      <c r="J33" t="s">
+        <v>184</v>
+      </c>
+      <c r="K33" t="s">
+        <v>185</v>
+      </c>
+      <c r="M33" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="N32" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="33" spans="3:14">
-      <c r="C33" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" t="s">
-        <v>48</v>
-      </c>
-      <c r="F33" t="s">
-        <v>100</v>
-      </c>
-      <c r="G33" t="s">
-        <v>100</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="I33" t="s">
-        <v>184</v>
-      </c>
-      <c r="J33" t="s">
-        <v>185</v>
-      </c>
-      <c r="K33" t="s">
-        <v>186</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="N33" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="3:14">
@@ -2273,31 +2225,31 @@
         <v>15</v>
       </c>
       <c r="D34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I34" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K34" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="3:14">
@@ -2305,95 +2257,89 @@
         <v>15</v>
       </c>
       <c r="D35" t="s">
+        <v>49</v>
+      </c>
+      <c r="F35" t="s">
+        <v>99</v>
+      </c>
+      <c r="G35" t="s">
+        <v>99</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I35" t="s">
+        <v>183</v>
+      </c>
+      <c r="J35" t="s">
+        <v>184</v>
+      </c>
+      <c r="K35" t="s">
+        <v>185</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="36" spans="3:14">
+      <c r="D36" t="s">
         <v>50</v>
       </c>
-      <c r="F35" t="s">
-        <v>100</v>
-      </c>
-      <c r="G35" t="s">
-        <v>100</v>
-      </c>
-      <c r="H35" s="2" t="s">
+      <c r="F36" t="s">
+        <v>99</v>
+      </c>
+      <c r="G36" t="s">
+        <v>99</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="I35" t="s">
-        <v>184</v>
-      </c>
-      <c r="J35" t="s">
-        <v>185</v>
-      </c>
-      <c r="K35" t="s">
-        <v>186</v>
-      </c>
-      <c r="M35" s="2" t="s">
+      <c r="I36" t="s">
+        <v>183</v>
+      </c>
+      <c r="J36" t="s">
+        <v>184</v>
+      </c>
+      <c r="K36" t="s">
+        <v>185</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="N35" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="36" spans="3:14">
-      <c r="C36" t="s">
-        <v>15</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="N36" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="37" spans="3:14">
+      <c r="D37" t="s">
         <v>51</v>
       </c>
-      <c r="F36" t="s">
-        <v>100</v>
-      </c>
-      <c r="G36" t="s">
-        <v>100</v>
-      </c>
-      <c r="H36" s="2" t="s">
+      <c r="F37" t="s">
+        <v>99</v>
+      </c>
+      <c r="G37" t="s">
+        <v>99</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="I36" t="s">
-        <v>184</v>
-      </c>
-      <c r="J36" t="s">
-        <v>185</v>
-      </c>
-      <c r="K36" t="s">
-        <v>186</v>
-      </c>
-      <c r="M36" s="2" t="s">
+      <c r="I37" t="s">
+        <v>183</v>
+      </c>
+      <c r="J37" t="s">
+        <v>184</v>
+      </c>
+      <c r="K37" t="s">
+        <v>185</v>
+      </c>
+      <c r="M37" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="N36" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="37" spans="3:14">
-      <c r="C37" t="s">
-        <v>15</v>
-      </c>
-      <c r="D37" t="s">
-        <v>52</v>
-      </c>
-      <c r="F37" t="s">
-        <v>100</v>
-      </c>
-      <c r="G37" t="s">
-        <v>100</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I37" t="s">
-        <v>184</v>
-      </c>
-      <c r="J37" t="s">
-        <v>185</v>
-      </c>
-      <c r="K37" t="s">
-        <v>186</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="N37" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="3:14">
@@ -2401,31 +2347,31 @@
         <v>15</v>
       </c>
       <c r="D38" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I38" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" spans="3:14">
@@ -2433,31 +2379,31 @@
         <v>15</v>
       </c>
       <c r="D39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I39" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J39" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="3:14">
@@ -2465,31 +2411,31 @@
         <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="3:14">
@@ -2497,63 +2443,60 @@
         <v>15</v>
       </c>
       <c r="D41" t="s">
+        <v>55</v>
+      </c>
+      <c r="F41" t="s">
+        <v>99</v>
+      </c>
+      <c r="G41" t="s">
+        <v>99</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I41" t="s">
+        <v>183</v>
+      </c>
+      <c r="J41" t="s">
+        <v>184</v>
+      </c>
+      <c r="K41" t="s">
+        <v>185</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="42" spans="3:14">
+      <c r="D42" t="s">
         <v>56</v>
       </c>
-      <c r="F41" t="s">
-        <v>100</v>
-      </c>
-      <c r="G41" t="s">
-        <v>100</v>
-      </c>
-      <c r="H41" s="2" t="s">
+      <c r="F42" t="s">
+        <v>99</v>
+      </c>
+      <c r="G42" t="s">
+        <v>99</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="I41" t="s">
-        <v>184</v>
-      </c>
-      <c r="J41" t="s">
-        <v>185</v>
-      </c>
-      <c r="K41" t="s">
-        <v>186</v>
-      </c>
-      <c r="M41" s="2" t="s">
+      <c r="I42" t="s">
+        <v>183</v>
+      </c>
+      <c r="J42" t="s">
+        <v>184</v>
+      </c>
+      <c r="K42" t="s">
+        <v>185</v>
+      </c>
+      <c r="M42" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="N41" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="42" spans="3:14">
-      <c r="C42" t="s">
-        <v>15</v>
-      </c>
-      <c r="D42" t="s">
-        <v>57</v>
-      </c>
-      <c r="F42" t="s">
-        <v>100</v>
-      </c>
-      <c r="G42" t="s">
-        <v>100</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="I42" t="s">
-        <v>184</v>
-      </c>
-      <c r="J42" t="s">
-        <v>185</v>
-      </c>
-      <c r="K42" t="s">
-        <v>186</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>227</v>
-      </c>
       <c r="N42" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="3:14">
@@ -2561,31 +2504,31 @@
         <v>15</v>
       </c>
       <c r="D43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I43" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J43" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K43" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" spans="3:14">
@@ -2593,31 +2536,31 @@
         <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I44" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J44" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K44" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="45" spans="3:14">
@@ -2625,31 +2568,31 @@
         <v>15</v>
       </c>
       <c r="D45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J45" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" spans="3:14">
@@ -2657,31 +2600,31 @@
         <v>15</v>
       </c>
       <c r="D46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I46" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K46" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="3:14">
@@ -2689,31 +2632,31 @@
         <v>15</v>
       </c>
       <c r="D47" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J47" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K47" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="48" spans="3:14">
@@ -2721,31 +2664,31 @@
         <v>15</v>
       </c>
       <c r="D48" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I48" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J48" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K48" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="49" spans="3:14">
@@ -2753,31 +2696,31 @@
         <v>15</v>
       </c>
       <c r="D49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I49" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J49" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K49" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="3:14">
@@ -2785,31 +2728,31 @@
         <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F50" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G50" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I50" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J50" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K50" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="51" spans="3:14">
@@ -2817,31 +2760,31 @@
         <v>15</v>
       </c>
       <c r="D51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I51" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J51" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K51" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" spans="3:14">
@@ -2849,31 +2792,31 @@
         <v>15</v>
       </c>
       <c r="D52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I52" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J52" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K52" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="3:14">
@@ -2881,31 +2824,31 @@
         <v>15</v>
       </c>
       <c r="D53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I53" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J53" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K53" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="54" spans="3:14">
@@ -2913,31 +2856,31 @@
         <v>15</v>
       </c>
       <c r="D54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I54" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J54" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K54" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="3:14">
@@ -2945,31 +2888,31 @@
         <v>15</v>
       </c>
       <c r="D55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J55" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K55" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="3:14">
@@ -2977,31 +2920,31 @@
         <v>15</v>
       </c>
       <c r="D56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I56" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J56" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K56" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="3:14">
@@ -3009,31 +2952,31 @@
         <v>15</v>
       </c>
       <c r="D57" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F57" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G57" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I57" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J57" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K57" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="3:14">
@@ -3041,31 +2984,31 @@
         <v>15</v>
       </c>
       <c r="D58" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I58" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J58" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K58" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="59" spans="3:14">
@@ -3073,31 +3016,31 @@
         <v>15</v>
       </c>
       <c r="D59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I59" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J59" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K59" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="60" spans="3:14">
@@ -3105,31 +3048,31 @@
         <v>15</v>
       </c>
       <c r="D60" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I60" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J60" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K60" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="61" spans="3:14">
@@ -3137,31 +3080,31 @@
         <v>15</v>
       </c>
       <c r="D61" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F61" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G61" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I61" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J61" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K61" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="3:14">
@@ -3169,31 +3112,31 @@
         <v>15</v>
       </c>
       <c r="D62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I62" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J62" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K62" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="3:14">
@@ -3201,31 +3144,31 @@
         <v>15</v>
       </c>
       <c r="D63" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I63" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J63" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K63" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="64" spans="3:14">
@@ -3233,31 +3176,31 @@
         <v>15</v>
       </c>
       <c r="D64" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G64" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I64" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J64" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K64" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="65" spans="3:14">
@@ -3265,31 +3208,31 @@
         <v>15</v>
       </c>
       <c r="D65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F65" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G65" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I65" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J65" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K65" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M65" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" spans="3:14">
@@ -3297,31 +3240,31 @@
         <v>15</v>
       </c>
       <c r="D66" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F66" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G66" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I66" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J66" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K66" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M66" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="67" spans="3:14">
@@ -3329,31 +3272,31 @@
         <v>15</v>
       </c>
       <c r="D67" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F67" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G67" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I67" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J67" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K67" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M67" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="N67" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="68" spans="3:14">
@@ -3361,31 +3304,31 @@
         <v>15</v>
       </c>
       <c r="D68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F68" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G68" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I68" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J68" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K68" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M68" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="69" spans="3:14">
@@ -3393,31 +3336,31 @@
         <v>15</v>
       </c>
       <c r="D69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F69" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G69" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I69" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J69" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K69" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M69" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="N69" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="70" spans="3:14">
@@ -3425,31 +3368,31 @@
         <v>15</v>
       </c>
       <c r="D70" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I70" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J70" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K70" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="71" spans="3:14">
@@ -3457,31 +3400,31 @@
         <v>15</v>
       </c>
       <c r="D71" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I71" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J71" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K71" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M71" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="N71" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="72" spans="3:14">
@@ -3489,31 +3432,31 @@
         <v>15</v>
       </c>
       <c r="D72" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F72" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G72" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I72" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J72" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K72" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="73" spans="3:14">
@@ -3521,31 +3464,31 @@
         <v>15</v>
       </c>
       <c r="D73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F73" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G73" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I73" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J73" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K73" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M73" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="N73" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="74" spans="3:14">
@@ -3553,31 +3496,31 @@
         <v>15</v>
       </c>
       <c r="D74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F74" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G74" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I74" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J74" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K74" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M74" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="N74" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="75" spans="3:14">
@@ -3585,31 +3528,31 @@
         <v>15</v>
       </c>
       <c r="D75" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F75" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G75" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I75" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J75" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K75" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M75" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N75" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="76" spans="3:14">
@@ -3617,31 +3560,31 @@
         <v>15</v>
       </c>
       <c r="D76" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F76" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G76" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I76" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J76" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K76" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M76" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="N76" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="77" spans="3:14">
@@ -3649,31 +3592,31 @@
         <v>15</v>
       </c>
       <c r="D77" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F77" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G77" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="I77" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J77" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K77" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M77" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="N77" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="78" spans="3:14">
@@ -3681,31 +3624,31 @@
         <v>15</v>
       </c>
       <c r="D78" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I78" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K78" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M78" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N78" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="79" spans="3:14">
@@ -3713,31 +3656,31 @@
         <v>15</v>
       </c>
       <c r="D79" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I79" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J79" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M79" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="N79" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="80" spans="3:14">
@@ -3745,31 +3688,31 @@
         <v>15</v>
       </c>
       <c r="D80" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I80" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J80" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K80" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M80" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N80" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="81" spans="3:14">
@@ -3777,31 +3720,31 @@
         <v>15</v>
       </c>
       <c r="D81" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="I81" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J81" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K81" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M81" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="N81" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="82" spans="3:14">
@@ -3809,31 +3752,31 @@
         <v>15</v>
       </c>
       <c r="D82" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F82" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G82" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I82" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J82" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K82" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M82" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="N82" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="83" spans="3:14">
@@ -3841,63 +3784,63 @@
         <v>15</v>
       </c>
       <c r="D83" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F83" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G83" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="I83" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J83" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K83" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M83" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="N83" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="84" spans="3:14">
       <c r="C84" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D84" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F84" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G84" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I84" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J84" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M84" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N84" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3948,208 +3891,208 @@
     <hyperlink ref="M16" r:id="rId44" location="geoid=0500000US39159"/>
     <hyperlink ref="N16" r:id="rId45"/>
     <hyperlink ref="H17" r:id="rId46"/>
-    <hyperlink ref="M17" r:id="rId47" location="geoid=0700000US390450695099999"/>
+    <hyperlink ref="M17" r:id="rId47" location="geoid=M100000US3902680"/>
     <hyperlink ref="N17" r:id="rId48"/>
     <hyperlink ref="H18" r:id="rId49"/>
-    <hyperlink ref="M18" r:id="rId50" location="geoid=0700000US390458020699999"/>
+    <hyperlink ref="M18" r:id="rId50" location="geoid=M100000US3903758"/>
     <hyperlink ref="N18" r:id="rId51"/>
     <hyperlink ref="H19" r:id="rId52"/>
-    <hyperlink ref="M19" r:id="rId53" location="geoid=0700000US390490692299999"/>
+    <hyperlink ref="M19" r:id="rId53" location="geoid=M100000US390450695099999"/>
     <hyperlink ref="N19" r:id="rId54"/>
     <hyperlink ref="H20" r:id="rId55"/>
-    <hyperlink ref="M20" r:id="rId56" location="geoid=0700000US390490944299999"/>
+    <hyperlink ref="M20" r:id="rId56" location="geoid=M100000US390458020699999"/>
     <hyperlink ref="N20" r:id="rId57"/>
     <hyperlink ref="H21" r:id="rId58"/>
-    <hyperlink ref="M21" r:id="rId59" location="geoid=0700000US390491611299999"/>
+    <hyperlink ref="M21" r:id="rId59" location="geoid=M100000US390490692299999"/>
     <hyperlink ref="N21" r:id="rId60"/>
     <hyperlink ref="H22" r:id="rId61"/>
-    <hyperlink ref="M22" r:id="rId62" location="geoid=0700000US390492828099999"/>
+    <hyperlink ref="M22" r:id="rId62" location="geoid=M100000US390490944299999"/>
     <hyperlink ref="N22" r:id="rId63"/>
     <hyperlink ref="H23" r:id="rId64"/>
-    <hyperlink ref="M23" r:id="rId65" location="geoid=0700000US390493777299999"/>
+    <hyperlink ref="M23" r:id="rId65" location="geoid=M100000US390491611299999"/>
     <hyperlink ref="N23" r:id="rId66"/>
     <hyperlink ref="H24" r:id="rId67"/>
-    <hyperlink ref="M24" r:id="rId68" location="geoid=0700000US390493861299999"/>
+    <hyperlink ref="M24" r:id="rId68" location="geoid=M100000US390492828099999"/>
     <hyperlink ref="N24" r:id="rId69"/>
     <hyperlink ref="H25" r:id="rId70"/>
-    <hyperlink ref="M25" r:id="rId71" location="geoid=0700000US390494641099999"/>
+    <hyperlink ref="M25" r:id="rId71" location="geoid=M100000US390493777299999"/>
     <hyperlink ref="N25" r:id="rId72"/>
     <hyperlink ref="H26" r:id="rId73"/>
-    <hyperlink ref="M26" r:id="rId74" location="geoid=0700000US390495006499999"/>
+    <hyperlink ref="M26" r:id="rId74" location="geoid=M100000US390493861299999"/>
     <hyperlink ref="N26" r:id="rId75"/>
     <hyperlink ref="H27" r:id="rId76"/>
-    <hyperlink ref="M27" r:id="rId77" location="geoid=0700000US390496184099999"/>
+    <hyperlink ref="M27" r:id="rId77" location="geoid=M100000US390494641099999"/>
     <hyperlink ref="N27" r:id="rId78"/>
     <hyperlink ref="H28" r:id="rId79"/>
-    <hyperlink ref="M28" r:id="rId80" location="geoid=0700000US390496297499999"/>
+    <hyperlink ref="M28" r:id="rId80" location="geoid=M100000US390495006499999"/>
     <hyperlink ref="N28" r:id="rId81"/>
     <hyperlink ref="H29" r:id="rId82"/>
-    <hyperlink ref="M29" r:id="rId83" location="geoid=0700000US390496457099999"/>
+    <hyperlink ref="M29" r:id="rId83" location="geoid=M100000US390496184099999"/>
     <hyperlink ref="N29" r:id="rId84"/>
     <hyperlink ref="H30" r:id="rId85"/>
-    <hyperlink ref="M30" r:id="rId86" location="geoid=0700000US390497771499999"/>
+    <hyperlink ref="M30" r:id="rId86" location="geoid=M100000US390496297499999"/>
     <hyperlink ref="N30" r:id="rId87"/>
     <hyperlink ref="H31" r:id="rId88"/>
-    <hyperlink ref="M31" r:id="rId89" location="geoid=0700000US390498124299999"/>
+    <hyperlink ref="M31" r:id="rId89" location="geoid=M100000US390496457099999"/>
     <hyperlink ref="N31" r:id="rId90"/>
     <hyperlink ref="H32" r:id="rId91"/>
-    <hyperlink ref="M32" r:id="rId92" location="geoid=0700000US390892569099999"/>
+    <hyperlink ref="M32" r:id="rId92" location="geoid=M100000US390497771499999"/>
     <hyperlink ref="N32" r:id="rId93"/>
     <hyperlink ref="H33" r:id="rId94"/>
-    <hyperlink ref="M33" r:id="rId95" location="geoid=0700000US390893141699999"/>
+    <hyperlink ref="M33" r:id="rId95" location="geoid=M100000US390498124299999"/>
     <hyperlink ref="N33" r:id="rId96"/>
     <hyperlink ref="H34" r:id="rId97"/>
-    <hyperlink ref="M34" r:id="rId98" location="geoid=0700000US391593904699999"/>
+    <hyperlink ref="M34" r:id="rId98" location="geoid=M100000US3905130"/>
     <hyperlink ref="N34" r:id="rId99"/>
     <hyperlink ref="H35" r:id="rId100"/>
-    <hyperlink ref="M35" r:id="rId101" location="geoid=1600000US3902680"/>
+    <hyperlink ref="M35" r:id="rId101" location="geoid=M100000US3906278"/>
     <hyperlink ref="N35" r:id="rId102"/>
     <hyperlink ref="H36" r:id="rId103"/>
-    <hyperlink ref="M36" r:id="rId104" location="geoid=1600000US3905130"/>
+    <hyperlink ref="M36" r:id="rId104" location="geoid=M100000US390892569099999"/>
     <hyperlink ref="N36" r:id="rId105"/>
     <hyperlink ref="H37" r:id="rId106"/>
-    <hyperlink ref="M37" r:id="rId107" location="geoid=1600000US3906278"/>
+    <hyperlink ref="M37" r:id="rId107" location="geoid=M100000US390893141699999"/>
     <hyperlink ref="N37" r:id="rId108"/>
     <hyperlink ref="H38" r:id="rId109"/>
-    <hyperlink ref="M38" r:id="rId110" location="geoid=1600000US3909890"/>
+    <hyperlink ref="M38" r:id="rId110" location="geoid=M100000US3909890"/>
     <hyperlink ref="N38" r:id="rId111"/>
     <hyperlink ref="H39" r:id="rId112"/>
-    <hyperlink ref="M39" r:id="rId113" location="geoid=1600000US3911332"/>
+    <hyperlink ref="M39" r:id="rId113" location="geoid=M100000US3911332"/>
     <hyperlink ref="N39" r:id="rId114"/>
     <hyperlink ref="H40" r:id="rId115"/>
-    <hyperlink ref="M40" r:id="rId116" location="geoid=1600000US3914184"/>
+    <hyperlink ref="M40" r:id="rId116" location="geoid=M100000US3914184"/>
     <hyperlink ref="N40" r:id="rId117"/>
     <hyperlink ref="H41" r:id="rId118"/>
-    <hyperlink ref="M41" r:id="rId119" location="geoid=1600000US3915070"/>
+    <hyperlink ref="M41" r:id="rId119" location="geoid=M100000US3915070"/>
     <hyperlink ref="N41" r:id="rId120"/>
     <hyperlink ref="H42" r:id="rId121"/>
-    <hyperlink ref="M42" r:id="rId122" location="geoid=1600000US3918000"/>
+    <hyperlink ref="M42" r:id="rId122" location="geoid=M100000US391593904699999"/>
     <hyperlink ref="N42" r:id="rId123"/>
     <hyperlink ref="H43" r:id="rId124"/>
-    <hyperlink ref="M43" r:id="rId125" location="geoid=1600000US3921434"/>
+    <hyperlink ref="M43" r:id="rId125" location="geoid=M100000US3918000"/>
     <hyperlink ref="N43" r:id="rId126"/>
     <hyperlink ref="H44" r:id="rId127"/>
-    <hyperlink ref="M44" r:id="rId128" location="geoid=1600000US3922694"/>
+    <hyperlink ref="M44" r:id="rId128" location="geoid=M100000US3921434"/>
     <hyperlink ref="N44" r:id="rId129"/>
     <hyperlink ref="H45" r:id="rId130"/>
-    <hyperlink ref="M45" r:id="rId131" location="geoid=1600000US3929106"/>
+    <hyperlink ref="M45" r:id="rId131" location="geoid=M100000US3922694"/>
     <hyperlink ref="N45" r:id="rId132"/>
     <hyperlink ref="H46" r:id="rId133"/>
-    <hyperlink ref="M46" r:id="rId134" location="geoid=1600000US3929148"/>
+    <hyperlink ref="M46" r:id="rId134" location="geoid=M100000US3929106"/>
     <hyperlink ref="N46" r:id="rId135"/>
     <hyperlink ref="H47" r:id="rId136"/>
-    <hyperlink ref="M47" r:id="rId137" location="geoid=1600000US3931304"/>
+    <hyperlink ref="M47" r:id="rId137" location="geoid=M100000US3929148"/>
     <hyperlink ref="N47" r:id="rId138"/>
     <hyperlink ref="H48" r:id="rId139"/>
-    <hyperlink ref="M48" r:id="rId140" location="geoid=1600000US3931402"/>
+    <hyperlink ref="M48" r:id="rId140" location="geoid=M100000US3931304"/>
     <hyperlink ref="N48" r:id="rId141"/>
     <hyperlink ref="H49" r:id="rId142"/>
-    <hyperlink ref="M49" r:id="rId143" location="geoid=1600000US3932592"/>
+    <hyperlink ref="M49" r:id="rId143" location="geoid=M100000US3931402"/>
     <hyperlink ref="N49" r:id="rId144"/>
     <hyperlink ref="H50" r:id="rId145"/>
-    <hyperlink ref="M50" r:id="rId146" location="geoid=1600000US3932606"/>
+    <hyperlink ref="M50" r:id="rId146" location="geoid=M100000US3932592"/>
     <hyperlink ref="N50" r:id="rId147"/>
     <hyperlink ref="H51" r:id="rId148"/>
-    <hyperlink ref="M51" r:id="rId149" location="geoid=1600000US3934748"/>
+    <hyperlink ref="M51" r:id="rId149" location="geoid=M100000US3932606"/>
     <hyperlink ref="N51" r:id="rId150"/>
     <hyperlink ref="H52" r:id="rId151"/>
-    <hyperlink ref="M52" r:id="rId152" location="geoid=1600000US3934790"/>
+    <hyperlink ref="M52" r:id="rId152" location="geoid=M100000US3934748"/>
     <hyperlink ref="N52" r:id="rId153"/>
     <hyperlink ref="H53" r:id="rId154"/>
-    <hyperlink ref="M53" r:id="rId155" location="geoid=1600000US3935476"/>
+    <hyperlink ref="M53" r:id="rId155" location="geoid=M100000US3934790"/>
     <hyperlink ref="N53" r:id="rId156"/>
     <hyperlink ref="H54" r:id="rId157"/>
-    <hyperlink ref="M54" r:id="rId158" location="geoid=1600000US3939340"/>
+    <hyperlink ref="M54" r:id="rId158" location="geoid=M100000US3935476"/>
     <hyperlink ref="N54" r:id="rId159"/>
     <hyperlink ref="H55" r:id="rId160"/>
-    <hyperlink ref="M55" r:id="rId161" location="geoid=1600000US3941720"/>
+    <hyperlink ref="M55" r:id="rId161" location="geoid=M100000US3939340"/>
     <hyperlink ref="N55" r:id="rId162"/>
     <hyperlink ref="H56" r:id="rId163"/>
-    <hyperlink ref="M56" r:id="rId164" location="geoid=1600000US3944086"/>
+    <hyperlink ref="M56" r:id="rId164" location="geoid=M100000US3941720"/>
     <hyperlink ref="N56" r:id="rId165"/>
     <hyperlink ref="H57" r:id="rId166"/>
-    <hyperlink ref="M57" r:id="rId167" location="geoid=1600000US3944674"/>
+    <hyperlink ref="M57" r:id="rId167" location="geoid=M100000US3944086"/>
     <hyperlink ref="N57" r:id="rId168"/>
     <hyperlink ref="H58" r:id="rId169"/>
-    <hyperlink ref="M58" r:id="rId170" location="geoid=1600000US3947474"/>
+    <hyperlink ref="M58" r:id="rId170" location="geoid=M100000US3944674"/>
     <hyperlink ref="N58" r:id="rId171"/>
     <hyperlink ref="H59" r:id="rId172"/>
-    <hyperlink ref="M59" r:id="rId173" location="geoid=1600000US3947754"/>
+    <hyperlink ref="M59" r:id="rId173" location="geoid=M100000US3947474"/>
     <hyperlink ref="N59" r:id="rId174"/>
     <hyperlink ref="H60" r:id="rId175"/>
-    <hyperlink ref="M60" r:id="rId176" location="geoid=1600000US3948160"/>
+    <hyperlink ref="M60" r:id="rId176" location="geoid=M100000US3947754"/>
     <hyperlink ref="N60" r:id="rId177"/>
     <hyperlink ref="H61" r:id="rId178"/>
-    <hyperlink ref="M61" r:id="rId179" location="geoid=1600000US3950862"/>
+    <hyperlink ref="M61" r:id="rId179" location="geoid=M100000US3948160"/>
     <hyperlink ref="N61" r:id="rId180"/>
     <hyperlink ref="H62" r:id="rId181"/>
-    <hyperlink ref="M62" r:id="rId182" location="geoid=1600000US3953046"/>
+    <hyperlink ref="M62" r:id="rId182" location="geoid=M100000US3950862"/>
     <hyperlink ref="N62" r:id="rId183"/>
     <hyperlink ref="H63" r:id="rId184"/>
-    <hyperlink ref="M63" r:id="rId185" location="geoid=1600000US3953102"/>
+    <hyperlink ref="M63" r:id="rId185" location="geoid=M100000US3953046"/>
     <hyperlink ref="N63" r:id="rId186"/>
     <hyperlink ref="H64" r:id="rId187"/>
-    <hyperlink ref="M64" r:id="rId188" location="geoid=1600000US3953970"/>
+    <hyperlink ref="M64" r:id="rId188" location="geoid=M100000US3953102"/>
     <hyperlink ref="N64" r:id="rId189"/>
     <hyperlink ref="H65" r:id="rId190"/>
-    <hyperlink ref="M65" r:id="rId191" location="geoid=1600000US3954040"/>
+    <hyperlink ref="M65" r:id="rId191" location="geoid=M100000US3953970"/>
     <hyperlink ref="N65" r:id="rId192"/>
     <hyperlink ref="H66" r:id="rId193"/>
-    <hyperlink ref="M66" r:id="rId194" location="geoid=1600000US3954866"/>
+    <hyperlink ref="M66" r:id="rId194" location="geoid=M100000US3954040"/>
     <hyperlink ref="N66" r:id="rId195"/>
     <hyperlink ref="H67" r:id="rId196"/>
-    <hyperlink ref="M67" r:id="rId197" location="geoid=1600000US3957862"/>
+    <hyperlink ref="M67" r:id="rId197" location="geoid=M100000US3954866"/>
     <hyperlink ref="N67" r:id="rId198"/>
     <hyperlink ref="H68" r:id="rId199"/>
-    <hyperlink ref="M68" r:id="rId200" location="geoid=1600000US3961112"/>
+    <hyperlink ref="M68" r:id="rId200" location="geoid=M100000US3957862"/>
     <hyperlink ref="N68" r:id="rId201"/>
     <hyperlink ref="H69" r:id="rId202"/>
-    <hyperlink ref="M69" r:id="rId203" location="geoid=1600000US3962498"/>
+    <hyperlink ref="M69" r:id="rId203" location="geoid=M100000US3961112"/>
     <hyperlink ref="N69" r:id="rId204"/>
     <hyperlink ref="H70" r:id="rId205"/>
-    <hyperlink ref="M70" r:id="rId206" location="geoid=1600000US3963030"/>
+    <hyperlink ref="M70" r:id="rId206" location="geoid=M100000US3962498"/>
     <hyperlink ref="N70" r:id="rId207"/>
     <hyperlink ref="H71" r:id="rId208"/>
-    <hyperlink ref="M71" r:id="rId209" location="geoid=1600000US3964486"/>
+    <hyperlink ref="M71" r:id="rId209" location="geoid=M100000US3963030"/>
     <hyperlink ref="N71" r:id="rId210"/>
     <hyperlink ref="H72" r:id="rId211"/>
-    <hyperlink ref="M72" r:id="rId212" location="geoid=1600000US3966390"/>
+    <hyperlink ref="M72" r:id="rId212" location="geoid=M100000US3964486"/>
     <hyperlink ref="N72" r:id="rId213"/>
     <hyperlink ref="H73" r:id="rId214"/>
-    <hyperlink ref="M73" r:id="rId215" location="geoid=1600000US3967440"/>
+    <hyperlink ref="M73" r:id="rId215" location="geoid=M100000US3966390"/>
     <hyperlink ref="N73" r:id="rId216"/>
     <hyperlink ref="H74" r:id="rId217"/>
-    <hyperlink ref="M74" r:id="rId218" location="geoid=1600000US3971976"/>
+    <hyperlink ref="M74" r:id="rId218" location="geoid=M100000US3967440"/>
     <hyperlink ref="N74" r:id="rId219"/>
     <hyperlink ref="H75" r:id="rId220"/>
-    <hyperlink ref="M75" r:id="rId221" location="geoid=1600000US3972977"/>
+    <hyperlink ref="M75" r:id="rId221" location="geoid=M100000US3971976"/>
     <hyperlink ref="N75" r:id="rId222"/>
     <hyperlink ref="H76" r:id="rId223"/>
-    <hyperlink ref="M76" r:id="rId224" location="geoid=1600000US3973068"/>
+    <hyperlink ref="M76" r:id="rId224" location="geoid=M100000US3972977"/>
     <hyperlink ref="N76" r:id="rId225"/>
     <hyperlink ref="H77" r:id="rId226"/>
-    <hyperlink ref="M77" r:id="rId227" location="geoid=1600000US3975602"/>
+    <hyperlink ref="M77" r:id="rId227" location="geoid=M100000US3973068"/>
     <hyperlink ref="N77" r:id="rId228"/>
     <hyperlink ref="H78" r:id="rId229"/>
-    <hyperlink ref="M78" r:id="rId230" location="geoid=1600000US3979002"/>
+    <hyperlink ref="M78" r:id="rId230" location="geoid=M100000US3975602"/>
     <hyperlink ref="N78" r:id="rId231"/>
     <hyperlink ref="H79" r:id="rId232"/>
-    <hyperlink ref="M79" r:id="rId233" location="geoid=1600000US3979100"/>
+    <hyperlink ref="M79" r:id="rId233" location="geoid=M100000US3979002"/>
     <hyperlink ref="N79" r:id="rId234"/>
     <hyperlink ref="H80" r:id="rId235"/>
-    <hyperlink ref="M80" r:id="rId236" location="geoid=1600000US3983342"/>
+    <hyperlink ref="M80" r:id="rId236" location="geoid=M100000US3979100"/>
     <hyperlink ref="N80" r:id="rId237"/>
     <hyperlink ref="H81" r:id="rId238"/>
-    <hyperlink ref="M81" r:id="rId239" location="geoid=1600000US3983580"/>
+    <hyperlink ref="M81" r:id="rId239" location="geoid=M100000US3983342"/>
     <hyperlink ref="N81" r:id="rId240"/>
     <hyperlink ref="H82" r:id="rId241"/>
-    <hyperlink ref="M82" r:id="rId242" location="geoid=1600000US3984742"/>
+    <hyperlink ref="M82" r:id="rId242" location="geoid=M100000US3983580"/>
     <hyperlink ref="N82" r:id="rId243"/>
     <hyperlink ref="H83" r:id="rId244"/>
-    <hyperlink ref="M83" r:id="rId245" location="geoid=1600000US3986604"/>
+    <hyperlink ref="M83" r:id="rId245" location="geoid=M100000US3984742"/>
     <hyperlink ref="N83" r:id="rId246"/>
     <hyperlink ref="H84" r:id="rId247"/>
-    <hyperlink ref="M84" r:id="rId248" location="geoid=M010000US001"/>
+    <hyperlink ref="M84" r:id="rId248" location="geoid=M100000US3986604"/>
     <hyperlink ref="N84" r:id="rId249"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>